<commit_message>
Dash DI - 30/04/2026
</commit_message>
<xml_diff>
--- a/Dados/Tratamento Exceções.xlsx
+++ b/Dados/Tratamento Exceções.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\Asset Management\Equipe\Lívia\HedgeCDI\Projeto-Hedge-CDI\Dados\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\Asset Management\Equipe\Emanuel\32.0-HedgeDI\Dados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5C01A51-9B00-415D-9709-4125F2179FE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47F9C9A6-7F5B-4533-B3A6-CB02A42D6346}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-1260" windowWidth="21840" windowHeight="13020" xr2:uid="{3663E241-9EA8-4CD8-9452-8494A5C65F2A}"/>
+    <workbookView xWindow="990" yWindow="900" windowWidth="23020" windowHeight="12220" xr2:uid="{3663E241-9EA8-4CD8-9452-8494A5C65F2A}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -28,6 +28,8 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -35,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="49">
   <si>
     <t>Código</t>
   </si>
@@ -148,7 +150,13 @@
     <t>PU Emissão</t>
   </si>
   <si>
+    <t>LFSN1800D4W</t>
+  </si>
+  <si>
     <t>LFSN210099R</t>
+  </si>
+  <si>
+    <t>PREFIXADA</t>
   </si>
   <si>
     <t>-</t>
@@ -182,16 +190,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -556,20 +558,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48B0AA01-3074-4CB8-8CE9-41A26084C332}">
-  <dimension ref="A1:I8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:I9"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="22.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.08984375" customWidth="1"/>
+    <col min="5" max="6" width="21.90625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.90625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -598,7 +597,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>26</v>
       </c>
@@ -621,61 +620,67 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>37</v>
       </c>
       <c r="B3" t="s">
         <v>39</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3">
+        <v>13.05</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>38</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="I3" s="1" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="B4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4">
-        <v>102.3</v>
-      </c>
-      <c r="D4" t="s">
-        <v>33</v>
-      </c>
-      <c r="F4" t="s">
-        <v>45</v>
-      </c>
-      <c r="G4" t="s">
-        <v>46</v>
-      </c>
-      <c r="I4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="D4" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B5" t="s">
         <v>9</v>
@@ -687,18 +692,18 @@
         <v>33</v>
       </c>
       <c r="F5" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G5" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="I5">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B6" t="s">
         <v>9</v>
@@ -710,18 +715,18 @@
         <v>33</v>
       </c>
       <c r="F6" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="I6">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B7" t="s">
         <v>9</v>
@@ -733,18 +738,18 @@
         <v>33</v>
       </c>
       <c r="F7" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G7" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="I7">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B8" t="s">
         <v>9</v>
@@ -756,17 +761,39 @@
         <v>33</v>
       </c>
       <c r="F8" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G8" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="I8">
         <v>1</v>
       </c>
     </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>46</v>
+      </c>
+      <c r="B9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9">
+        <v>102.3</v>
+      </c>
+      <c r="D9" t="s">
+        <v>33</v>
+      </c>
+      <c r="F9" t="s">
+        <v>47</v>
+      </c>
+      <c r="G9" t="s">
+        <v>48</v>
+      </c>
+      <c r="I9">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
@@ -774,16 +801,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18106D39-0059-4512-9229-3DA7948252BC}">
   <dimension ref="A1:H16"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="8" width="22.5703125" bestFit="1" customWidth="1"/>
-  </cols>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -809,7 +829,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -832,7 +852,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -852,7 +872,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>15</v>
       </c>
@@ -878,7 +898,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -904,7 +924,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>17</v>
       </c>
@@ -930,7 +950,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>18</v>
       </c>
@@ -956,7 +976,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -982,7 +1002,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>20</v>
       </c>
@@ -1008,7 +1028,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>21</v>
       </c>
@@ -1034,7 +1054,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>22</v>
       </c>
@@ -1060,7 +1080,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>23</v>
       </c>
@@ -1086,7 +1106,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>24</v>
       </c>
@@ -1112,7 +1132,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>25</v>
       </c>
@@ -1138,7 +1158,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>26</v>
       </c>
@@ -1164,7 +1184,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>27</v>
       </c>

</xml_diff>

<commit_message>
Dash CDI - 09/06/2026
</commit_message>
<xml_diff>
--- a/Dados/Tratamento Exceções.xlsx
+++ b/Dados/Tratamento Exceções.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\Asset Management\Equipe\Lívia\HedgeCDI\Projeto-Hedge-CDI\Dados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92AFF39A-3BC4-4352-ACA7-C3CCA71993E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CA601F6-25DC-4265-BD29-EC6B7DBEBD0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="20370" yWindow="-1260" windowWidth="21840" windowHeight="13020" xr2:uid="{3663E241-9EA8-4CD8-9452-8494A5C65F2A}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="51">
   <si>
     <t>Código</t>
   </si>
@@ -660,9 +660,7 @@
       <c r="D4" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="E4" s="1" t="s">
-        <v>39</v>
-      </c>
+      <c r="E4" s="1"/>
       <c r="F4" s="1" t="s">
         <v>39</v>
       </c>

</xml_diff>